<commit_message>
Simplify the CMO spend report to three categories
Drops the network-cost and other-payments lines from the summary and the
detail sheet; both amounts now sit inside the remaining balance, so the
report reads as received, spent on three things, and what is left.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01XVAJSqts3cNZjAS2RnUVZY
</commit_message>
<xml_diff>
--- a/informe/gasto_wallet.xlsx
+++ b/informe/gasto_wallet.xlsx
@@ -12,7 +12,7 @@
     <sheet name="Pagos a KOLs" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detalle'!$A$1:$F$36</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Detalle'!$A$1:$F$35</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -23,7 +23,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="7">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -62,11 +62,6 @@
       <name val="Arial"/>
       <color rgb="00595959"/>
       <sz val="10"/>
-    </font>
-    <font>
-      <name val="Arial"/>
-      <color rgb="000000FF"/>
-      <sz val="11"/>
     </font>
   </fonts>
   <fills count="4">
@@ -118,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -129,7 +124,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="4" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -245,12 +239,12 @@
           </spPr>
           <cat>
             <numRef>
-              <f>'Resumen'!$A$7:$A$11</f>
+              <f>'Resumen'!$A$7:$A$9</f>
             </numRef>
           </cat>
           <val>
             <numRef>
-              <f>'Resumen'!$B$7:$B$11</f>
+              <f>'Resumen'!$B$7:$B$9</f>
             </numRef>
           </val>
         </ser>
@@ -603,7 +597,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C21"/>
+  <dimension ref="A1:C18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -689,81 +683,52 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>Otros pagos</t>
-        </is>
-      </c>
-      <c r="B10" s="7">
-        <f>SUMIF(Detalle!B:B,A10,Detalle!D:D)</f>
-        <v>41.65</v>
+      <c r="A10" s="8" t="inlineStr">
+        <is>
+          <t>TOTAL GASTADO</t>
+        </is>
+      </c>
+      <c r="B10" s="9">
+        <f>SUM(B7:B9)</f>
+        <v>18677.62</v>
         <v/>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>Coste de mover el dinero</t>
-        </is>
-      </c>
-      <c r="B11" s="8" t="n">
-        <v>232.54</v>
-      </c>
-    </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
-        <is>
-          <t>TOTAL GASTADO</t>
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Queda disponible</t>
         </is>
       </c>
       <c r="B12" s="10">
-        <f>SUM(B7:B11)</f>
-        <v>18951.81</v>
+        <f>B4-B10</f>
+        <v>4322.38</v>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
-        <is>
-          <t>Queda disponible</t>
-        </is>
-      </c>
-      <c r="B14" s="11">
-        <f>B4-B12</f>
-        <v>4048.19</v>
-        <v/>
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Notas</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Importes en dólares. Los pagos se hicieron en USDC, que vale 1 dólar.</t>
+        </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr">
-        <is>
-          <t>Notas</t>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>El detalle de cada operación, con enlace para verla, está en la pestaña «Detalle».</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
-        <is>
-          <t>Importes en dólares. Los pagos se hicieron en USDC, que vale 1 dólar.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="inlineStr">
-        <is>
-          <t>«Coste de mover el dinero» es lo que cuesta cada operación en la red y pasar fondos de Ethereum a Base.</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>El detalle de cada operación, con enlace para verla, está en la pestaña «Detalle».</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="2" t="inlineStr">
         <is>
           <t>Fuente: registro público de Ethereum y Base (etherscan.io y basescan.org).</t>
         </is>
@@ -781,7 +746,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F38"/>
+  <dimension ref="A1:F37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -825,1069 +790,1039 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="11" t="inlineStr">
         <is>
           <t>2026-07-02</t>
         </is>
       </c>
-      <c r="B2" s="12" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>Campañas rally.fun</t>
         </is>
       </c>
-      <c r="C2" s="12" t="inlineStr">
+      <c r="C2" s="11" t="inlineStr">
         <is>
           <t>rally.fun (contrato de campaña)</t>
         </is>
       </c>
-      <c r="D2" s="13" t="n">
+      <c r="D2" s="12" t="n">
         <v>5000</v>
       </c>
-      <c r="E2" s="12" t="inlineStr">
+      <c r="E2" s="11" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="F2" s="14" t="inlineStr">
+      <c r="F2" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="11" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="B3" s="12" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Campañas rally.fun</t>
         </is>
       </c>
-      <c r="C3" s="12" t="inlineStr">
+      <c r="C3" s="11" t="inlineStr">
         <is>
           <t>rally.fun (contrato de campaña)</t>
         </is>
       </c>
-      <c r="D3" s="13" t="n">
+      <c r="D3" s="12" t="n">
         <v>1000</v>
       </c>
-      <c r="E3" s="12" t="inlineStr">
+      <c r="E3" s="11" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="F3" s="14" t="inlineStr">
+      <c r="F3" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="11" t="inlineStr">
         <is>
           <t>2026-07-10</t>
         </is>
       </c>
-      <c r="B4" s="12" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Campañas rally.fun</t>
         </is>
       </c>
-      <c r="C4" s="12" t="inlineStr">
+      <c r="C4" s="11" t="inlineStr">
         <is>
           <t>rally.fun (fondeo de campañas)</t>
         </is>
       </c>
-      <c r="D4" s="13" t="n">
+      <c r="D4" s="12" t="n">
         <v>2050</v>
       </c>
-      <c r="E4" s="12" t="inlineStr">
+      <c r="E4" s="11" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="F4" s="14" t="inlineStr">
+      <c r="F4" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>2026-07-15</t>
         </is>
       </c>
-      <c r="B5" s="12" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Campañas rally.fun</t>
         </is>
       </c>
-      <c r="C5" s="12" t="inlineStr">
+      <c r="C5" s="11" t="inlineStr">
         <is>
           <t>rally.fun (fondeo de campañas)</t>
         </is>
       </c>
-      <c r="D5" s="13" t="n">
+      <c r="D5" s="12" t="n">
         <v>1010</v>
       </c>
-      <c r="E5" s="12" t="inlineStr">
+      <c r="E5" s="11" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="F5" s="14" t="inlineStr">
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>2026-07-24</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Campañas rally.fun</t>
         </is>
       </c>
-      <c r="C6" s="12" t="inlineStr">
+      <c r="C6" s="11" t="inlineStr">
         <is>
           <t>rally.fun (fondeo de campañas)</t>
         </is>
       </c>
-      <c r="D6" s="13" t="n">
+      <c r="D6" s="12" t="n">
         <v>1050</v>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E6" s="11" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="F6" s="14" t="inlineStr">
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
-      <c r="B7" s="12" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Campañas rally.fun</t>
         </is>
       </c>
-      <c r="C7" s="12" t="inlineStr">
+      <c r="C7" s="11" t="inlineStr">
         <is>
           <t>rally.fun (fondeo de campañas)</t>
         </is>
       </c>
-      <c r="D7" s="13" t="n">
+      <c r="D7" s="12" t="n">
         <v>3010</v>
       </c>
-      <c r="E7" s="12" t="inlineStr">
+      <c r="E7" s="11" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="F7" s="14" t="inlineStr">
+      <c r="F7" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Pagos a KOLs</t>
         </is>
       </c>
-      <c r="C8" s="12" t="inlineStr">
+      <c r="C8" s="11" t="inlineStr">
         <is>
           <t>*javi🥥️.eth</t>
         </is>
       </c>
-      <c r="D8" s="13" t="n">
+      <c r="D8" s="12" t="n">
         <v>400</v>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E8" s="11" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="F8" s="14" t="inlineStr">
+      <c r="F8" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B9" s="12" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Pagos a KOLs</t>
         </is>
       </c>
-      <c r="C9" s="12" t="inlineStr">
+      <c r="C9" s="11" t="inlineStr">
         <is>
           <t>oeiras.base.eth</t>
         </is>
       </c>
-      <c r="D9" s="13" t="n">
+      <c r="D9" s="12" t="n">
         <v>400</v>
       </c>
-      <c r="E9" s="12" t="inlineStr">
+      <c r="E9" s="11" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="F9" s="14" t="inlineStr">
+      <c r="F9" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B10" s="12" t="inlineStr">
+      <c r="B10" s="11" t="inlineStr">
         <is>
           <t>Pagos a KOLs</t>
         </is>
       </c>
-      <c r="C10" s="12" t="inlineStr">
+      <c r="C10" s="11" t="inlineStr">
         <is>
           <t>grebby.base.eth</t>
         </is>
       </c>
-      <c r="D10" s="13" t="n">
+      <c r="D10" s="12" t="n">
         <v>500</v>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E10" s="11" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="F10" s="14" t="inlineStr">
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
-      <c r="B11" s="12" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Pagos a KOLs</t>
         </is>
       </c>
-      <c r="C11" s="12" t="inlineStr">
+      <c r="C11" s="11" t="inlineStr">
         <is>
           <t>0x36df9ebc…11ac</t>
         </is>
       </c>
-      <c r="D11" s="13" t="n">
+      <c r="D11" s="12" t="n">
         <v>400</v>
       </c>
-      <c r="E11" s="12" t="inlineStr">
+      <c r="E11" s="11" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="F11" s="14" t="inlineStr">
+      <c r="F11" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="B12" s="12" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Pagos a KOLs</t>
         </is>
       </c>
-      <c r="C12" s="12" t="inlineStr">
+      <c r="C12" s="11" t="inlineStr">
         <is>
           <t>caominh.base.eth</t>
         </is>
       </c>
-      <c r="D12" s="13" t="n">
+      <c r="D12" s="12" t="n">
         <v>400</v>
       </c>
-      <c r="E12" s="12" t="inlineStr">
+      <c r="E12" s="11" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="F12" s="14" t="inlineStr">
+      <c r="F12" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="B13" s="12" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Pagos a KOLs</t>
         </is>
       </c>
-      <c r="C13" s="12" t="inlineStr">
+      <c r="C13" s="11" t="inlineStr">
         <is>
           <t>0xbd04be7d…cfde</t>
         </is>
       </c>
-      <c r="D13" s="13" t="n">
+      <c r="D13" s="12" t="n">
         <v>400</v>
       </c>
-      <c r="E13" s="12" t="inlineStr">
+      <c r="E13" s="11" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="F13" s="14" t="inlineStr">
+      <c r="F13" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="B14" s="12" t="inlineStr">
+      <c r="B14" s="11" t="inlineStr">
         <is>
           <t>Pagos a KOLs</t>
         </is>
       </c>
-      <c r="C14" s="12" t="inlineStr">
+      <c r="C14" s="11" t="inlineStr">
         <is>
           <t>0x391e81fb…62d8</t>
         </is>
       </c>
-      <c r="D14" s="13" t="n">
+      <c r="D14" s="12" t="n">
         <v>400</v>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="E14" s="11" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="F14" s="14" t="inlineStr">
+      <c r="F14" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="B15" s="12" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Pagos a KOLs</t>
         </is>
       </c>
-      <c r="C15" s="12" t="inlineStr">
+      <c r="C15" s="11" t="inlineStr">
         <is>
           <t>0xc766e44b…b46c</t>
         </is>
       </c>
-      <c r="D15" s="13" t="n">
+      <c r="D15" s="12" t="n">
         <v>200</v>
       </c>
-      <c r="E15" s="12" t="inlineStr">
+      <c r="E15" s="11" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="F15" s="14" t="inlineStr">
+      <c r="F15" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="11" t="inlineStr">
         <is>
           <t>Pagos a KOLs</t>
         </is>
       </c>
-      <c r="C16" s="12" t="inlineStr">
+      <c r="C16" s="11" t="inlineStr">
         <is>
           <t>seyra.base.eth</t>
         </is>
       </c>
-      <c r="D16" s="13" t="n">
+      <c r="D16" s="12" t="n">
         <v>200</v>
       </c>
-      <c r="E16" s="12" t="inlineStr">
+      <c r="E16" s="11" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="F16" s="14" t="inlineStr">
+      <c r="F16" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="12" t="inlineStr">
+      <c r="A17" s="11" t="inlineStr">
         <is>
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>Pagos a KOLs</t>
         </is>
       </c>
-      <c r="C17" s="12" t="inlineStr">
+      <c r="C17" s="11" t="inlineStr">
         <is>
           <t>seyra.base.eth</t>
         </is>
       </c>
-      <c r="D17" s="13" t="n">
+      <c r="D17" s="12" t="n">
         <v>200</v>
       </c>
-      <c r="E17" s="12" t="inlineStr">
+      <c r="E17" s="11" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="F17" s="14" t="inlineStr">
+      <c r="F17" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="12" t="inlineStr">
+      <c r="A18" s="11" t="inlineStr">
         <is>
           <t>2026-07-17</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B18" s="11" t="inlineStr">
         <is>
           <t>Pagos a KOLs</t>
         </is>
       </c>
-      <c r="C18" s="12" t="inlineStr">
+      <c r="C18" s="11" t="inlineStr">
         <is>
           <t>0x01882087…5ae2</t>
         </is>
       </c>
-      <c r="D18" s="13" t="n">
+      <c r="D18" s="12" t="n">
         <v>400</v>
       </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="E18" s="11" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="F18" s="14" t="inlineStr">
+      <c r="F18" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="12" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Pagos a KOLs</t>
         </is>
       </c>
-      <c r="C19" s="12" t="inlineStr">
+      <c r="C19" s="11" t="inlineStr">
         <is>
           <t>0xb124e658…c0b9</t>
         </is>
       </c>
-      <c r="D19" s="13" t="n">
+      <c r="D19" s="12" t="n">
         <v>500</v>
       </c>
-      <c r="E19" s="12" t="inlineStr">
+      <c r="E19" s="11" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="F19" s="14" t="inlineStr">
+      <c r="F19" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="12" t="inlineStr">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>2026-08-18</t>
         </is>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B20" s="11" t="inlineStr">
         <is>
           <t>Pagos a KOLs</t>
         </is>
       </c>
-      <c r="C20" s="12" t="inlineStr">
+      <c r="C20" s="11" t="inlineStr">
         <is>
           <t>0xcc8fff36…780d</t>
         </is>
       </c>
-      <c r="D20" s="13" t="n">
+      <c r="D20" s="12" t="n">
         <v>200</v>
       </c>
-      <c r="E20" s="12" t="inlineStr">
+      <c r="E20" s="11" t="inlineStr">
         <is>
           <t>Base</t>
         </is>
       </c>
-      <c r="F20" s="14" t="inlineStr">
+      <c r="F20" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="12" t="inlineStr">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>NFTs</t>
         </is>
       </c>
-      <c r="C21" s="12" t="inlineStr">
+      <c r="C21" s="11" t="inlineStr">
         <is>
           <t>Compra de NFT</t>
         </is>
       </c>
-      <c r="D21" s="13" t="n">
+      <c r="D21" s="12" t="n">
         <v>31.12</v>
       </c>
-      <c r="E21" s="12" t="inlineStr">
+      <c r="E21" s="11" t="inlineStr">
         <is>
           <t>Ethereum</t>
         </is>
       </c>
-      <c r="F21" s="14" t="inlineStr">
+      <c r="F21" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="12" t="inlineStr">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B22" s="11" t="inlineStr">
         <is>
           <t>NFTs</t>
         </is>
       </c>
-      <c r="C22" s="12" t="inlineStr">
+      <c r="C22" s="11" t="inlineStr">
         <is>
           <t>Compra de NFT</t>
         </is>
       </c>
-      <c r="D22" s="13" t="n">
+      <c r="D22" s="12" t="n">
         <v>31.69</v>
       </c>
-      <c r="E22" s="12" t="inlineStr">
+      <c r="E22" s="11" t="inlineStr">
         <is>
           <t>Ethereum</t>
         </is>
       </c>
-      <c r="F22" s="14" t="inlineStr">
+      <c r="F22" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="12" t="inlineStr">
+      <c r="A23" s="11" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>NFTs</t>
         </is>
       </c>
-      <c r="C23" s="12" t="inlineStr">
+      <c r="C23" s="11" t="inlineStr">
         <is>
           <t>Compra de NFT</t>
         </is>
       </c>
-      <c r="D23" s="13" t="n">
+      <c r="D23" s="12" t="n">
         <v>30.37</v>
       </c>
-      <c r="E23" s="12" t="inlineStr">
+      <c r="E23" s="11" t="inlineStr">
         <is>
           <t>Ethereum</t>
         </is>
       </c>
-      <c r="F23" s="14" t="inlineStr">
+      <c r="F23" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="12" t="inlineStr">
+      <c r="A24" s="11" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="B24" s="11" t="inlineStr">
         <is>
           <t>NFTs</t>
         </is>
       </c>
-      <c r="C24" s="12" t="inlineStr">
+      <c r="C24" s="11" t="inlineStr">
         <is>
           <t>Compra de NFT</t>
         </is>
       </c>
-      <c r="D24" s="13" t="n">
+      <c r="D24" s="12" t="n">
         <v>31.15</v>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="E24" s="11" t="inlineStr">
         <is>
           <t>Ethereum</t>
         </is>
       </c>
-      <c r="F24" s="14" t="inlineStr">
+      <c r="F24" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="12" t="inlineStr">
+      <c r="A25" s="11" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>NFTs</t>
         </is>
       </c>
-      <c r="C25" s="12" t="inlineStr">
+      <c r="C25" s="11" t="inlineStr">
         <is>
           <t>Compra de NFT</t>
         </is>
       </c>
-      <c r="D25" s="13" t="n">
+      <c r="D25" s="12" t="n">
         <v>33.39</v>
       </c>
-      <c r="E25" s="12" t="inlineStr">
+      <c r="E25" s="11" t="inlineStr">
         <is>
           <t>Ethereum</t>
         </is>
       </c>
-      <c r="F25" s="14" t="inlineStr">
+      <c r="F25" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="12" t="inlineStr">
+      <c r="A26" s="11" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B26" s="12" t="inlineStr">
+      <c r="B26" s="11" t="inlineStr">
         <is>
           <t>NFTs</t>
         </is>
       </c>
-      <c r="C26" s="12" t="inlineStr">
+      <c r="C26" s="11" t="inlineStr">
         <is>
           <t>Compra de NFT</t>
         </is>
       </c>
-      <c r="D26" s="13" t="n">
+      <c r="D26" s="12" t="n">
         <v>39.13</v>
       </c>
-      <c r="E26" s="12" t="inlineStr">
+      <c r="E26" s="11" t="inlineStr">
         <is>
           <t>Ethereum</t>
         </is>
       </c>
-      <c r="F26" s="14" t="inlineStr">
+      <c r="F26" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="27">
-      <c r="A27" s="12" t="inlineStr">
+      <c r="A27" s="11" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>NFTs</t>
         </is>
       </c>
-      <c r="C27" s="12" t="inlineStr">
+      <c r="C27" s="11" t="inlineStr">
         <is>
           <t>Compra de NFT</t>
         </is>
       </c>
-      <c r="D27" s="13" t="n">
+      <c r="D27" s="12" t="n">
         <v>40.86</v>
       </c>
-      <c r="E27" s="12" t="inlineStr">
+      <c r="E27" s="11" t="inlineStr">
         <is>
           <t>Ethereum</t>
         </is>
       </c>
-      <c r="F27" s="14" t="inlineStr">
+      <c r="F27" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="28">
-      <c r="A28" s="12" t="inlineStr">
+      <c r="A28" s="11" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B28" s="12" t="inlineStr">
+      <c r="B28" s="11" t="inlineStr">
         <is>
           <t>NFTs</t>
         </is>
       </c>
-      <c r="C28" s="12" t="inlineStr">
+      <c r="C28" s="11" t="inlineStr">
         <is>
           <t>Compra de NFT</t>
         </is>
       </c>
-      <c r="D28" s="13" t="n">
+      <c r="D28" s="12" t="n">
         <v>41.16</v>
       </c>
-      <c r="E28" s="12" t="inlineStr">
+      <c r="E28" s="11" t="inlineStr">
         <is>
           <t>Ethereum</t>
         </is>
       </c>
-      <c r="F28" s="14" t="inlineStr">
+      <c r="F28" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="12" t="inlineStr">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>NFTs</t>
         </is>
       </c>
-      <c r="C29" s="12" t="inlineStr">
+      <c r="C29" s="11" t="inlineStr">
         <is>
           <t>Compra de NFT</t>
         </is>
       </c>
-      <c r="D29" s="13" t="n">
+      <c r="D29" s="12" t="n">
         <v>35.4</v>
       </c>
-      <c r="E29" s="12" t="inlineStr">
+      <c r="E29" s="11" t="inlineStr">
         <is>
           <t>Ethereum</t>
         </is>
       </c>
-      <c r="F29" s="14" t="inlineStr">
+      <c r="F29" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="30">
-      <c r="A30" s="12" t="inlineStr">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B30" s="11" t="inlineStr">
         <is>
           <t>NFTs</t>
         </is>
       </c>
-      <c r="C30" s="12" t="inlineStr">
+      <c r="C30" s="11" t="inlineStr">
         <is>
           <t>Compra de NFT</t>
         </is>
       </c>
-      <c r="D30" s="13" t="n">
+      <c r="D30" s="12" t="n">
         <v>35.4</v>
       </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="E30" s="11" t="inlineStr">
         <is>
           <t>Ethereum</t>
         </is>
       </c>
-      <c r="F30" s="14" t="inlineStr">
+      <c r="F30" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="12" t="inlineStr">
+      <c r="A31" s="11" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B31" s="12" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>NFTs</t>
         </is>
       </c>
-      <c r="C31" s="12" t="inlineStr">
+      <c r="C31" s="11" t="inlineStr">
         <is>
           <t>Compra de NFT</t>
         </is>
       </c>
-      <c r="D31" s="13" t="n">
+      <c r="D31" s="12" t="n">
         <v>41.65</v>
       </c>
-      <c r="E31" s="12" t="inlineStr">
+      <c r="E31" s="11" t="inlineStr">
         <is>
           <t>Ethereum</t>
         </is>
       </c>
-      <c r="F31" s="14" t="inlineStr">
+      <c r="F31" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="32">
-      <c r="A32" s="12" t="inlineStr">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B32" s="12" t="inlineStr">
+      <c r="B32" s="11" t="inlineStr">
         <is>
           <t>NFTs</t>
         </is>
       </c>
-      <c r="C32" s="12" t="inlineStr">
+      <c r="C32" s="11" t="inlineStr">
         <is>
           <t>Compra de NFT</t>
         </is>
       </c>
-      <c r="D32" s="13" t="n">
+      <c r="D32" s="12" t="n">
         <v>39.57</v>
       </c>
-      <c r="E32" s="12" t="inlineStr">
+      <c r="E32" s="11" t="inlineStr">
         <is>
           <t>Ethereum</t>
         </is>
       </c>
-      <c r="F32" s="14" t="inlineStr">
+      <c r="F32" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="33">
-      <c r="A33" s="12" t="inlineStr">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
+      <c r="B33" s="11" t="inlineStr">
         <is>
           <t>NFTs</t>
         </is>
       </c>
-      <c r="C33" s="12" t="inlineStr">
+      <c r="C33" s="11" t="inlineStr">
         <is>
           <t>Compra de NFT</t>
         </is>
       </c>
-      <c r="D33" s="13" t="n">
+      <c r="D33" s="12" t="n">
         <v>38.92</v>
       </c>
-      <c r="E33" s="12" t="inlineStr">
+      <c r="E33" s="11" t="inlineStr">
         <is>
           <t>Ethereum</t>
         </is>
       </c>
-      <c r="F33" s="14" t="inlineStr">
+      <c r="F33" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="12" t="inlineStr">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t>2026-07-07</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
+      <c r="B34" s="11" t="inlineStr">
         <is>
           <t>NFTs</t>
         </is>
       </c>
-      <c r="C34" s="12" t="inlineStr">
+      <c r="C34" s="11" t="inlineStr">
         <is>
           <t>Compra de NFT</t>
         </is>
       </c>
-      <c r="D34" s="13" t="n">
+      <c r="D34" s="12" t="n">
         <v>47.9</v>
       </c>
-      <c r="E34" s="12" t="inlineStr">
+      <c r="E34" s="11" t="inlineStr">
         <is>
           <t>Ethereum</t>
         </is>
       </c>
-      <c r="F34" s="14" t="inlineStr">
+      <c r="F34" s="13" t="inlineStr">
         <is>
           <t>Abrir</t>
         </is>
       </c>
     </row>
     <row r="35">
-      <c r="A35" s="12" t="inlineStr">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>2026-07-12</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B35" s="11" t="inlineStr">
         <is>
           <t>NFTs</t>
         </is>
       </c>
-      <c r="C35" s="12" t="inlineStr">
+      <c r="C35" s="11" t="inlineStr">
         <is>
           <t>Compra de NFT</t>
         </is>
       </c>
-      <c r="D35" s="13" t="n">
+      <c r="D35" s="12" t="n">
         <v>439.91</v>
       </c>
-      <c r="E35" s="12" t="inlineStr">
+      <c r="E35" s="11" t="inlineStr">
         <is>
           <t>Ethereum</t>
         </is>
       </c>
-      <c r="F35" s="14" t="inlineStr">
-        <is>
-          <t>Abrir</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="12" t="inlineStr">
-        <is>
-          <t>2026-07-03</t>
-        </is>
-      </c>
-      <c r="B36" s="12" t="inlineStr">
-        <is>
-          <t>Otros pagos</t>
-        </is>
-      </c>
-      <c r="C36" s="12" t="inlineStr">
-        <is>
-          <t>0x599873fC…45D4</t>
-        </is>
-      </c>
-      <c r="D36" s="13" t="n">
-        <v>41.65</v>
-      </c>
-      <c r="E36" s="12" t="inlineStr">
-        <is>
-          <t>Ethereum</t>
-        </is>
-      </c>
-      <c r="F36" s="14" t="inlineStr">
-        <is>
-          <t>Abrir</t>
-        </is>
-      </c>
-    </row>
-    <row r="38">
-      <c r="C38" s="9" t="inlineStr">
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>Abrir</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="C37" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="D38" s="10">
-        <f>SUM(D2:D36)</f>
-        <v>18719.27</v>
+      <c r="D37" s="9">
+        <f>SUM(D2:D35)</f>
+        <v>18677.62</v>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:F36"/>
+  <autoFilter ref="A1:F35"/>
   <hyperlinks>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F2" r:id="rId1"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F3" r:id="rId2"/>
@@ -1923,7 +1858,6 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F33" r:id="rId32"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F34" r:id="rId33"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F35" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F36" r:id="rId35"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1981,238 +1915,238 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="11" t="inlineStr">
         <is>
           <t>grebby.base.eth</t>
         </is>
       </c>
-      <c r="B5" s="12" t="n">
+      <c r="B5" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C5" s="13" t="n">
+      <c r="C5" s="12" t="n">
         <v>500</v>
       </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="D5" s="11" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="11" t="inlineStr">
         <is>
           <t>0xb124e658…c0b9</t>
         </is>
       </c>
-      <c r="B6" s="12" t="n">
+      <c r="B6" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C6" s="13" t="n">
+      <c r="C6" s="12" t="n">
         <v>500</v>
       </c>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="D6" s="11" t="inlineStr">
         <is>
           <t>2026-08-03</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="11" t="inlineStr">
         <is>
           <t>*javi🥥️.eth</t>
         </is>
       </c>
-      <c r="B7" s="12" t="n">
+      <c r="B7" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C7" s="13" t="n">
+      <c r="C7" s="12" t="n">
         <v>400</v>
       </c>
-      <c r="D7" s="12" t="inlineStr">
+      <c r="D7" s="11" t="inlineStr">
         <is>
           <t>2026-07-03</t>
         </is>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="11" t="inlineStr">
         <is>
           <t>oeiras.base.eth</t>
         </is>
       </c>
-      <c r="B8" s="12" t="n">
+      <c r="B8" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C8" s="13" t="n">
+      <c r="C8" s="12" t="n">
         <v>400</v>
       </c>
-      <c r="D8" s="12" t="inlineStr">
+      <c r="D8" s="11" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+      <c r="A9" s="11" t="inlineStr">
         <is>
           <t>0x36df9ebc…11ac</t>
         </is>
       </c>
-      <c r="B9" s="12" t="n">
+      <c r="B9" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C9" s="13" t="n">
+      <c r="C9" s="12" t="n">
         <v>400</v>
       </c>
-      <c r="D9" s="12" t="inlineStr">
+      <c r="D9" s="11" t="inlineStr">
         <is>
           <t>2026-07-06</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="12" t="inlineStr">
+      <c r="A10" s="11" t="inlineStr">
         <is>
           <t>caominh.base.eth</t>
         </is>
       </c>
-      <c r="B10" s="12" t="n">
+      <c r="B10" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C10" s="13" t="n">
+      <c r="C10" s="12" t="n">
         <v>400</v>
       </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="D10" s="11" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="12" t="inlineStr">
+      <c r="A11" s="11" t="inlineStr">
         <is>
           <t>0xbd04be7d…cfde</t>
         </is>
       </c>
-      <c r="B11" s="12" t="n">
+      <c r="B11" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C11" s="13" t="n">
+      <c r="C11" s="12" t="n">
         <v>400</v>
       </c>
-      <c r="D11" s="12" t="inlineStr">
+      <c r="D11" s="11" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="12" t="inlineStr">
+      <c r="A12" s="11" t="inlineStr">
         <is>
           <t>0x391e81fb…62d8</t>
         </is>
       </c>
-      <c r="B12" s="12" t="n">
+      <c r="B12" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C12" s="13" t="n">
+      <c r="C12" s="12" t="n">
         <v>400</v>
       </c>
-      <c r="D12" s="12" t="inlineStr">
+      <c r="D12" s="11" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="12" t="inlineStr">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>seyra.base.eth</t>
         </is>
       </c>
-      <c r="B13" s="12" t="n">
+      <c r="B13" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="C13" s="13" t="n">
+      <c r="C13" s="12" t="n">
         <v>400</v>
       </c>
-      <c r="D13" s="12" t="inlineStr">
+      <c r="D13" s="11" t="inlineStr">
         <is>
           <t>2026-07-09, 2026-07-17</t>
         </is>
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="12" t="inlineStr">
+      <c r="A14" s="11" t="inlineStr">
         <is>
           <t>0x01882087…5ae2</t>
         </is>
       </c>
-      <c r="B14" s="12" t="n">
+      <c r="B14" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C14" s="13" t="n">
+      <c r="C14" s="12" t="n">
         <v>400</v>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D14" s="11" t="inlineStr">
         <is>
           <t>2026-07-17</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="12" t="inlineStr">
+      <c r="A15" s="11" t="inlineStr">
         <is>
           <t>0xc766e44b…b46c</t>
         </is>
       </c>
-      <c r="B15" s="12" t="n">
+      <c r="B15" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C15" s="13" t="n">
+      <c r="C15" s="12" t="n">
         <v>200</v>
       </c>
-      <c r="D15" s="12" t="inlineStr">
+      <c r="D15" s="11" t="inlineStr">
         <is>
           <t>2026-07-09</t>
         </is>
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="12" t="inlineStr">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>0xcc8fff36…780d</t>
         </is>
       </c>
-      <c r="B16" s="12" t="n">
+      <c r="B16" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="C16" s="13" t="n">
+      <c r="C16" s="12" t="n">
         <v>200</v>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="D16" s="11" t="inlineStr">
         <is>
           <t>2026-08-18</t>
         </is>
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="9" t="inlineStr">
+      <c r="A18" s="8" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B18" s="9">
+      <c r="B18" s="8">
         <f>SUM(B5:B16)</f>
         <v>13</v>
         <v/>
       </c>
-      <c r="C18" s="10">
+      <c r="C18" s="9">
         <f>SUM(C5:C16)</f>
         <v>4600</v>
         <v/>
       </c>
-      <c r="D18" s="15" t="inlineStr">
+      <c r="D18" s="14" t="inlineStr">
         <is>
           <t> </t>
         </is>

</xml_diff>